<commit_message>
Updated models and drugs
</commit_message>
<xml_diff>
--- a/data/Drug_list_112524.xlsx
+++ b/data/Drug_list_112524.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tim\Documents\Silverman\BEN-SHALOM\Hartwell\NetPyne\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/romanbaravalle/M1_NEURON_paper/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16E4C99-724E-4003-8F70-10EED3A5AE45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC123EAB-C545-BE47-A75F-70AFE30A19EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9996" yWindow="0" windowWidth="34560" windowHeight="25296" xr2:uid="{A3335644-D6CD-434C-BD76-9E6C48E66893}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34560" windowHeight="20340" xr2:uid="{A3335644-D6CD-434C-BD76-9E6C48E66893}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="73">
   <si>
     <t>Drug</t>
   </si>
@@ -240,13 +240,28 @@
   </si>
   <si>
     <t>Increase K+ current -- increase gbar K channel across board</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>One sodium channel</t>
+  </si>
+  <si>
+    <t>One calcium channel</t>
+  </si>
+  <si>
+    <t>One potassium channel</t>
+  </si>
+  <si>
+    <t>One GABA, one AMPA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,16 +290,35 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -292,23 +326,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -327,7 +392,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -643,61 +708,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41742F95-3161-4880-BCE5-74ACAB02B981}">
-  <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32.88671875" customWidth="1"/>
-    <col min="3" max="3" width="94.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="94.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="E1" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="E2" s="9"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="11" t="s">
         <v>57</v>
       </c>
       <c r="E3" s="2"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -712,7 +779,7 @@
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -727,37 +794,37 @@
       </c>
       <c r="E5" s="2"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="7" t="s">
         <v>58</v>
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="7" t="s">
         <v>59</v>
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -772,7 +839,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -787,22 +854,22 @@
       </c>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -817,7 +884,7 @@
       </c>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -832,7 +899,7 @@
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -847,37 +914,37 @@
       </c>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="7" t="s">
         <v>66</v>
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="11" t="s">
         <v>66</v>
       </c>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>13</v>
       </c>
@@ -892,37 +959,37 @@
       </c>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="7" t="s">
         <v>63</v>
       </c>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="7" t="s">
         <v>67</v>
       </c>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
@@ -937,7 +1004,7 @@
       </c>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
@@ -952,7 +1019,7 @@
       </c>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>18</v>
       </c>
@@ -967,7 +1034,7 @@
       </c>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>19</v>
       </c>
@@ -982,7 +1049,7 @@
       </c>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
@@ -997,7 +1064,7 @@
       </c>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>21</v>
       </c>
@@ -1012,7 +1079,7 @@
       </c>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>22</v>
       </c>
@@ -1027,35 +1094,55 @@
       </c>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D26" s="3" t="s">
+      <c r="D26" s="7" t="s">
         <v>64</v>
       </c>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="7" t="s">
         <v>65</v>
       </c>
       <c r="E27" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C31" s="13" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="C32" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C33" s="13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C34" s="13" t="s">
+        <v>71</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>